<commit_message>
Fix: Setup LFS and clean up large files
</commit_message>
<xml_diff>
--- a/TMD regions annotation - full 451 1.xlsx
+++ b/TMD regions annotation - full 451 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XN\du-an-dung-chung\Methyl-GW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XN\du-an-dung-chung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A70F17-70C5-49D5-AD78-8E0A4EAC92FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8092498-07C8-4D06-9C7C-D4AD1D3F80A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E5475C7F-0BD2-46B2-ACB0-D317CA76E7C1}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="20730" windowHeight="11040" xr2:uid="{E5475C7F-0BD2-46B2-ACB0-D317CA76E7C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="862">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="861">
   <si>
     <t>Region</t>
   </si>
@@ -1954,9 +1954,6 @@
   </si>
   <si>
     <t>TMD_335</t>
-  </si>
-  <si>
-    <t>MARCH11</t>
   </si>
   <si>
     <t>TMD_336</t>
@@ -2667,7 +2664,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2685,6 +2682,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11081,8 +11081,8 @@
       <c r="E336" s="3">
         <v>16180455</v>
       </c>
-      <c r="F336" s="1" t="s">
-        <v>640</v>
+      <c r="F336" s="7">
+        <v>40603</v>
       </c>
       <c r="G336" t="str">
         <f t="shared" si="5"/>
@@ -11091,7 +11091,7 @@
     </row>
     <row r="337" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A337" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>13</v>
@@ -11106,7 +11106,7 @@
         <v>40681354</v>
       </c>
       <c r="F337" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="G337" t="str">
         <f t="shared" si="5"/>
@@ -11115,7 +11115,7 @@
     </row>
     <row r="338" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A338" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>7</v>
@@ -11130,7 +11130,7 @@
         <v>72594977</v>
       </c>
       <c r="F338" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="G338" t="str">
         <f t="shared" si="5"/>
@@ -11139,7 +11139,7 @@
     </row>
     <row r="339" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A339" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>7</v>
@@ -11154,7 +11154,7 @@
         <v>72715515</v>
       </c>
       <c r="F339" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="G339" t="str">
         <f t="shared" si="5"/>
@@ -11163,7 +11163,7 @@
     </row>
     <row r="340" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A340" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>13</v>
@@ -11178,7 +11178,7 @@
         <v>76249811</v>
       </c>
       <c r="F340" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="G340" t="str">
         <f t="shared" si="5"/>
@@ -11187,7 +11187,7 @@
     </row>
     <row r="341" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A341" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B341" s="1" t="s">
         <v>13</v>
@@ -11202,7 +11202,7 @@
         <v>134374869</v>
       </c>
       <c r="F341" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="G341" t="str">
         <f t="shared" si="5"/>
@@ -11211,7 +11211,7 @@
     </row>
     <row r="342" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A342" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>13</v>
@@ -11226,7 +11226,7 @@
         <v>140801091</v>
       </c>
       <c r="F342" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="G342" t="str">
         <f t="shared" si="5"/>
@@ -11235,7 +11235,7 @@
     </row>
     <row r="343" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A343" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>20</v>
@@ -11250,7 +11250,7 @@
         <v>140893043</v>
       </c>
       <c r="F343" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G343" t="str">
         <f t="shared" si="5"/>
@@ -11259,7 +11259,7 @@
     </row>
     <row r="344" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A344" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>7</v>
@@ -11274,7 +11274,7 @@
         <v>153862397</v>
       </c>
       <c r="F344" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G344" t="str">
         <f t="shared" si="5"/>
@@ -11283,7 +11283,7 @@
     </row>
     <row r="345" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A345" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>17</v>
@@ -11298,7 +11298,7 @@
         <v>168307354</v>
       </c>
       <c r="F345" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="G345" t="str">
         <f t="shared" si="5"/>
@@ -11307,7 +11307,7 @@
     </row>
     <row r="346" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A346" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>7</v>
@@ -11322,7 +11322,7 @@
         <v>172673044</v>
       </c>
       <c r="F346" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="G346" t="str">
         <f t="shared" si="5"/>
@@ -11331,7 +11331,7 @@
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A347" s="1" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B347" s="1" t="s">
         <v>7</v>
@@ -11346,7 +11346,7 @@
         <v>177411831</v>
       </c>
       <c r="F347" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G347" t="str">
         <f t="shared" si="5"/>
@@ -11355,7 +11355,7 @@
     </row>
     <row r="348" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A348" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>17</v>
@@ -11370,7 +11370,7 @@
         <v>178004060</v>
       </c>
       <c r="F348" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="G348" t="str">
         <f t="shared" si="5"/>
@@ -11379,7 +11379,7 @@
     </row>
     <row r="349" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A349" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B349" s="1" t="s">
         <v>7</v>
@@ -11394,7 +11394,7 @@
         <v>179894413</v>
       </c>
       <c r="F349" s="1" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G349" t="str">
         <f t="shared" si="5"/>
@@ -11403,7 +11403,7 @@
     </row>
     <row r="350" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A350" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>13</v>
@@ -11418,7 +11418,7 @@
         <v>180486766</v>
       </c>
       <c r="F350" s="1" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="G350" t="str">
         <f t="shared" si="5"/>
@@ -11427,7 +11427,7 @@
     </row>
     <row r="351" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A351" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>20</v>
@@ -11442,7 +11442,7 @@
         <v>112073518</v>
       </c>
       <c r="F351" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G351" t="str">
         <f t="shared" si="5"/>
@@ -11451,7 +11451,7 @@
     </row>
     <row r="352" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A352" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>20</v>
@@ -11466,7 +11466,7 @@
         <v>115152575</v>
       </c>
       <c r="F352" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="G352" t="str">
         <f t="shared" si="5"/>
@@ -11475,13 +11475,13 @@
     </row>
     <row r="353" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A353" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B353" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C353" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D353" s="3">
         <v>1378651</v>
@@ -11490,7 +11490,7 @@
         <v>1378856</v>
       </c>
       <c r="F353" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="G353" t="str">
         <f t="shared" si="5"/>
@@ -11499,13 +11499,13 @@
     </row>
     <row r="354" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A354" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B354" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C354" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D354" s="3">
         <v>6003907</v>
@@ -11514,7 +11514,7 @@
         <v>6004299</v>
       </c>
       <c r="F354" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="G354" t="str">
         <f t="shared" si="5"/>
@@ -11523,13 +11523,13 @@
     </row>
     <row r="355" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A355" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C355" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D355" s="3">
         <v>10417573</v>
@@ -11538,7 +11538,7 @@
         <v>10417778</v>
       </c>
       <c r="F355" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="G355" t="str">
         <f t="shared" si="5"/>
@@ -11547,13 +11547,13 @@
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A356" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C356" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D356" s="3">
         <v>10421371</v>
@@ -11562,7 +11562,7 @@
         <v>10421804</v>
       </c>
       <c r="F356" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="G356" t="str">
         <f t="shared" si="5"/>
@@ -11571,13 +11571,13 @@
     </row>
     <row r="357" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A357" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D357" s="3">
         <v>19691729</v>
@@ -11586,7 +11586,7 @@
         <v>19692173</v>
       </c>
       <c r="F357" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G357" t="str">
         <f t="shared" si="5"/>
@@ -11595,13 +11595,13 @@
     </row>
     <row r="358" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A358" s="1" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B358" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C358" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D358" s="3">
         <v>30131360</v>
@@ -11610,7 +11610,7 @@
         <v>30131614</v>
       </c>
       <c r="F358" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="G358" t="str">
         <f t="shared" si="5"/>
@@ -11619,13 +11619,13 @@
     </row>
     <row r="359" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A359" s="1" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B359" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C359" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D359" s="3">
         <v>32157425</v>
@@ -11634,7 +11634,7 @@
         <v>32157687</v>
       </c>
       <c r="F359" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="G359" t="str">
         <f t="shared" si="5"/>
@@ -11643,13 +11643,13 @@
     </row>
     <row r="360" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A360" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B360" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C360" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D360" s="3">
         <v>36253025</v>
@@ -11658,7 +11658,7 @@
         <v>36253261</v>
       </c>
       <c r="F360" s="1" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="G360" t="str">
         <f t="shared" si="5"/>
@@ -11667,13 +11667,13 @@
     </row>
     <row r="361" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A361" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C361" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D361" s="3">
         <v>38683076</v>
@@ -11682,7 +11682,7 @@
         <v>38683301</v>
       </c>
       <c r="F361" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="G361" t="str">
         <f t="shared" si="5"/>
@@ -11691,13 +11691,13 @@
     </row>
     <row r="362" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A362" s="1" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B362" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C362" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D362" s="3">
         <v>41341406</v>
@@ -11706,7 +11706,7 @@
         <v>41341751</v>
       </c>
       <c r="F362" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="G362" t="str">
         <f t="shared" si="5"/>
@@ -11715,13 +11715,13 @@
     </row>
     <row r="363" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A363" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B363" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C363" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D363" s="3">
         <v>41528448</v>
@@ -11730,7 +11730,7 @@
         <v>41528958</v>
       </c>
       <c r="F363" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G363" t="str">
         <f t="shared" si="5"/>
@@ -11739,13 +11739,13 @@
     </row>
     <row r="364" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A364" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C364" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D364" s="3">
         <v>42072032</v>
@@ -11754,7 +11754,7 @@
         <v>42072648</v>
       </c>
       <c r="F364" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G364" t="str">
         <f t="shared" si="5"/>
@@ -11763,13 +11763,13 @@
     </row>
     <row r="365" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A365" s="1" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B365" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C365" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D365" s="3">
         <v>50818148</v>
@@ -11778,7 +11778,7 @@
         <v>50818365</v>
       </c>
       <c r="F365" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="G365" t="str">
         <f t="shared" si="5"/>
@@ -11787,13 +11787,13 @@
     </row>
     <row r="366" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A366" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C366" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D366" s="3">
         <v>56716258</v>
@@ -11802,7 +11802,7 @@
         <v>56716537</v>
       </c>
       <c r="F366" s="1" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="G366" t="str">
         <f t="shared" si="5"/>
@@ -11811,13 +11811,13 @@
     </row>
     <row r="367" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A367" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B367" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C367" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D367" s="3">
         <v>85476087</v>
@@ -11826,7 +11826,7 @@
         <v>85476330</v>
       </c>
       <c r="F367" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="G367" t="str">
         <f t="shared" si="5"/>
@@ -11835,13 +11835,13 @@
     </row>
     <row r="368" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A368" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B368" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C368" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D368" s="3">
         <v>85477013</v>
@@ -11850,7 +11850,7 @@
         <v>85477284</v>
       </c>
       <c r="F368" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="G368" t="str">
         <f t="shared" si="5"/>
@@ -11859,13 +11859,13 @@
     </row>
     <row r="369" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A369" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B369" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C369" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D369" s="3">
         <v>106433875</v>
@@ -11874,7 +11874,7 @@
         <v>106434297</v>
       </c>
       <c r="F369" s="1" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G369" t="str">
         <f t="shared" si="5"/>
@@ -11883,13 +11883,13 @@
     </row>
     <row r="370" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A370" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B370" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C370" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D370" s="3">
         <v>137814472</v>
@@ -11898,7 +11898,7 @@
         <v>137814861</v>
       </c>
       <c r="F370" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="G370" t="str">
         <f t="shared" si="5"/>
@@ -11907,13 +11907,13 @@
     </row>
     <row r="371" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A371" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B371" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C371" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D371" s="3">
         <v>143234754</v>
@@ -11922,7 +11922,7 @@
         <v>143234818</v>
       </c>
       <c r="F371" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="G371" t="str">
         <f t="shared" si="5"/>
@@ -11931,13 +11931,13 @@
     </row>
     <row r="372" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A372" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B372" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C372" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D372" s="3">
         <v>143234931</v>
@@ -11946,7 +11946,7 @@
         <v>143235067</v>
       </c>
       <c r="F372" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="G372" t="str">
         <f t="shared" si="5"/>
@@ -11955,13 +11955,13 @@
     </row>
     <row r="373" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A373" s="1" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C373" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D373" s="3">
         <v>151004536</v>
@@ -11970,7 +11970,7 @@
         <v>151004727</v>
       </c>
       <c r="F373" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="G373" t="str">
         <f t="shared" si="5"/>
@@ -11979,13 +11979,13 @@
     </row>
     <row r="374" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A374" s="1" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B374" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C374" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D374" s="3">
         <v>163817971</v>
@@ -11994,7 +11994,7 @@
         <v>163818242</v>
       </c>
       <c r="F374" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="G374" t="str">
         <f t="shared" si="5"/>
@@ -12003,13 +12003,13 @@
     </row>
     <row r="375" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A375" s="1" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B375" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C375" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D375" s="3">
         <v>170494223</v>
@@ -12018,7 +12018,7 @@
         <v>170494454</v>
       </c>
       <c r="F375" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G375" t="str">
         <f t="shared" si="5"/>
@@ -12027,13 +12027,13 @@
     </row>
     <row r="376" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A376" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B376" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C376" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D376" s="3">
         <v>170494241</v>
@@ -12042,7 +12042,7 @@
         <v>170494362</v>
       </c>
       <c r="F376" s="1" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G376" t="str">
         <f t="shared" si="5"/>
@@ -12051,13 +12051,13 @@
     </row>
     <row r="377" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A377" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B377" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C377" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D377" s="3">
         <v>3247630</v>
@@ -12066,7 +12066,7 @@
         <v>3247751</v>
       </c>
       <c r="F377" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G377" t="str">
         <f t="shared" si="5"/>
@@ -12075,13 +12075,13 @@
     </row>
     <row r="378" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A378" s="1" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B378" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C378" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D378" s="3">
         <v>391393</v>
@@ -12090,7 +12090,7 @@
         <v>391545</v>
       </c>
       <c r="F378" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G378" t="str">
         <f t="shared" si="5"/>
@@ -12099,13 +12099,13 @@
     </row>
     <row r="379" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A379" s="1" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B379" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C379" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D379" s="3">
         <v>641090</v>
@@ -12114,7 +12114,7 @@
         <v>641403</v>
       </c>
       <c r="F379" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="G379" t="str">
         <f t="shared" si="5"/>
@@ -12123,13 +12123,13 @@
     </row>
     <row r="380" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A380" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B380" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C380" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D380" s="3">
         <v>1263580</v>
@@ -12138,7 +12138,7 @@
         <v>1263840</v>
       </c>
       <c r="F380" s="1" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="G380" t="str">
         <f t="shared" si="5"/>
@@ -12147,13 +12147,13 @@
     </row>
     <row r="381" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A381" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B381" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C381" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D381" s="3">
         <v>4859593</v>
@@ -12162,7 +12162,7 @@
         <v>4859779</v>
       </c>
       <c r="F381" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G381" t="str">
         <f t="shared" si="5"/>
@@ -12171,13 +12171,13 @@
     </row>
     <row r="382" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A382" s="1" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B382" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C382" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D382" s="3">
         <v>27196417</v>
@@ -12186,7 +12186,7 @@
         <v>27196625</v>
       </c>
       <c r="F382" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G382" t="str">
         <f t="shared" si="5"/>
@@ -12195,13 +12195,13 @@
     </row>
     <row r="383" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A383" s="1" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B383" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C383" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D383" s="3">
         <v>27206024</v>
@@ -12210,7 +12210,7 @@
         <v>27206238</v>
       </c>
       <c r="F383" s="1" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G383" t="str">
         <f t="shared" si="5"/>
@@ -12219,13 +12219,13 @@
     </row>
     <row r="384" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A384" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B384" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C384" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D384" s="3">
         <v>27260129</v>
@@ -12234,7 +12234,7 @@
         <v>27260467</v>
       </c>
       <c r="F384" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="G384" t="str">
         <f t="shared" si="5"/>
@@ -12243,13 +12243,13 @@
     </row>
     <row r="385" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A385" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B385" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C385" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D385" s="3">
         <v>27283472</v>
@@ -12258,7 +12258,7 @@
         <v>27283676</v>
       </c>
       <c r="F385" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G385" t="str">
         <f t="shared" si="5"/>
@@ -12267,13 +12267,13 @@
     </row>
     <row r="386" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A386" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B386" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C386" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D386" s="3">
         <v>29603208</v>
@@ -12282,7 +12282,7 @@
         <v>29603408</v>
       </c>
       <c r="F386" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G386" t="str">
         <f t="shared" si="5"/>
@@ -12291,13 +12291,13 @@
     </row>
     <row r="387" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A387" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B387" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C387" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D387" s="3">
         <v>29605641</v>
@@ -12306,7 +12306,7 @@
         <v>29606290</v>
       </c>
       <c r="F387" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G387" t="str">
         <f t="shared" ref="G387:G450" si="6">C387&amp;":"&amp;D387&amp;"-"&amp;E387</f>
@@ -12315,13 +12315,13 @@
     </row>
     <row r="388" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A388" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B388" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C388" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D388" s="3">
         <v>35293620</v>
@@ -12330,7 +12330,7 @@
         <v>35293984</v>
       </c>
       <c r="F388" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G388" t="str">
         <f t="shared" si="6"/>
@@ -12339,13 +12339,13 @@
     </row>
     <row r="389" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A389" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B389" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C389" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D389" s="3">
         <v>35297390</v>
@@ -12354,7 +12354,7 @@
         <v>35297595</v>
       </c>
       <c r="F389" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G389" t="str">
         <f t="shared" si="6"/>
@@ -12363,13 +12363,13 @@
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A390" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B390" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C390" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D390" s="3">
         <v>55248872</v>
@@ -12378,7 +12378,7 @@
         <v>55249088</v>
       </c>
       <c r="F390" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G390" t="str">
         <f t="shared" si="6"/>
@@ -12387,13 +12387,13 @@
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A391" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B391" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C391" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D391" s="3">
         <v>67016137</v>
@@ -12402,7 +12402,7 @@
         <v>67016255</v>
       </c>
       <c r="F391" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G391" t="str">
         <f t="shared" si="6"/>
@@ -12411,13 +12411,13 @@
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A392" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B392" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C392" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D392" s="3">
         <v>70111546</v>
@@ -12426,7 +12426,7 @@
         <v>70111758</v>
       </c>
       <c r="F392" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G392" t="str">
         <f t="shared" si="6"/>
@@ -12435,13 +12435,13 @@
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A393" s="1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B393" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C393" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D393" s="3">
         <v>71802022</v>
@@ -12450,7 +12450,7 @@
         <v>71802283</v>
       </c>
       <c r="F393" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G393" t="str">
         <f t="shared" si="6"/>
@@ -12459,13 +12459,13 @@
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A394" s="1" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B394" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C394" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D394" s="3">
         <v>97361441</v>
@@ -12474,7 +12474,7 @@
         <v>97361635</v>
       </c>
       <c r="F394" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G394" t="str">
         <f t="shared" si="6"/>
@@ -12483,13 +12483,13 @@
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A395" s="1" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B395" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C395" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D395" s="3">
         <v>97361747</v>
@@ -12498,7 +12498,7 @@
         <v>97361815</v>
       </c>
       <c r="F395" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G395" t="str">
         <f t="shared" si="6"/>
@@ -12507,13 +12507,13 @@
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A396" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B396" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C396" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D396" s="3">
         <v>121950117</v>
@@ -12522,7 +12522,7 @@
         <v>121950351</v>
       </c>
       <c r="F396" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G396" t="str">
         <f t="shared" si="6"/>
@@ -12531,13 +12531,13 @@
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A397" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B397" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C397" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D397" s="3">
         <v>121950621</v>
@@ -12546,7 +12546,7 @@
         <v>121950800</v>
       </c>
       <c r="F397" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G397" t="str">
         <f t="shared" si="6"/>
@@ -12555,13 +12555,13 @@
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A398" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="B398" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C398" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D398" s="3">
         <v>127991841</v>
@@ -12570,7 +12570,7 @@
         <v>127992012</v>
       </c>
       <c r="F398" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G398" t="str">
         <f t="shared" si="6"/>
@@ -12579,13 +12579,13 @@
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A399" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B399" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C399" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D399" s="3">
         <v>127992202</v>
@@ -12594,7 +12594,7 @@
         <v>127992439</v>
       </c>
       <c r="F399" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G399" t="str">
         <f t="shared" si="6"/>
@@ -12603,13 +12603,13 @@
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A400" s="1" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B400" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C400" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D400" s="3">
         <v>150655279</v>
@@ -12618,7 +12618,7 @@
         <v>150655530</v>
       </c>
       <c r="F400" s="1" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="G400" t="str">
         <f t="shared" si="6"/>
@@ -12627,13 +12627,13 @@
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A401" s="1" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B401" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C401" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D401" s="3">
         <v>154409595</v>
@@ -12642,7 +12642,7 @@
         <v>154409721</v>
       </c>
       <c r="F401" s="1" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="G401" t="str">
         <f t="shared" si="6"/>
@@ -12651,13 +12651,13 @@
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A402" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B402" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C402" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D402" s="3">
         <v>156400843</v>
@@ -12666,7 +12666,7 @@
         <v>156401092</v>
       </c>
       <c r="F402" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G402" t="str">
         <f t="shared" si="6"/>
@@ -12675,13 +12675,13 @@
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A403" s="1" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B403" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C403" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D403" s="3">
         <v>156798401</v>
@@ -12690,7 +12690,7 @@
         <v>156798722</v>
       </c>
       <c r="F403" s="1" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="G403" t="str">
         <f t="shared" si="6"/>
@@ -12699,13 +12699,13 @@
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A404" s="1" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B404" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C404" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D404" s="3">
         <v>156810853</v>
@@ -12714,7 +12714,7 @@
         <v>156811073</v>
       </c>
       <c r="F404" s="1" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="G404" t="str">
         <f t="shared" si="6"/>
@@ -12723,13 +12723,13 @@
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A405" s="1" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B405" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C405" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D405" s="3">
         <v>156811251</v>
@@ -12738,7 +12738,7 @@
         <v>156811441</v>
       </c>
       <c r="F405" s="1" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="G405" t="str">
         <f t="shared" si="6"/>
@@ -12747,13 +12747,13 @@
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A406" s="1" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B406" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C406" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D406" s="3">
         <v>157478278</v>
@@ -12762,7 +12762,7 @@
         <v>157478491</v>
       </c>
       <c r="F406" s="1" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="G406" t="str">
         <f t="shared" si="6"/>
@@ -12771,13 +12771,13 @@
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A407" s="1" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B407" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C407" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D407" s="3">
         <v>97361294</v>
@@ -12786,7 +12786,7 @@
         <v>97361446</v>
       </c>
       <c r="F407" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G407" t="str">
         <f t="shared" si="6"/>
@@ -12795,13 +12795,13 @@
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A408" s="1" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B408" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C408" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D408" s="3">
         <v>27135828</v>
@@ -12810,7 +12810,7 @@
         <v>27135898</v>
       </c>
       <c r="F408" s="1" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="G408" t="str">
         <f t="shared" si="6"/>
@@ -12819,13 +12819,13 @@
     </row>
     <row r="409" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A409" s="1" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B409" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C409" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D409" s="3">
         <v>50343867</v>
@@ -12834,7 +12834,7 @@
         <v>50343961</v>
       </c>
       <c r="F409" s="1" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="G409" t="str">
         <f t="shared" si="6"/>
@@ -12843,13 +12843,13 @@
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A410" s="1" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B410" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C410" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D410" s="3">
         <v>686980</v>
@@ -12858,7 +12858,7 @@
         <v>687150</v>
       </c>
       <c r="F410" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="G410" t="str">
         <f t="shared" si="6"/>
@@ -12867,13 +12867,13 @@
     </row>
     <row r="411" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A411" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B411" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C411" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D411" s="3">
         <v>687364</v>
@@ -12882,7 +12882,7 @@
         <v>687587</v>
       </c>
       <c r="F411" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="G411" t="str">
         <f t="shared" si="6"/>
@@ -12891,13 +12891,13 @@
     </row>
     <row r="412" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A412" s="1" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B412" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C412" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D412" s="3">
         <v>3549494</v>
@@ -12915,13 +12915,13 @@
     </row>
     <row r="413" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A413" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B413" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C413" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D413" s="3">
         <v>10588882</v>
@@ -12930,7 +12930,7 @@
         <v>10589207</v>
       </c>
       <c r="F413" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="G413" t="str">
         <f t="shared" si="6"/>
@@ -12939,13 +12939,13 @@
     </row>
     <row r="414" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A414" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B414" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C414" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D414" s="3">
         <v>20375577</v>
@@ -12954,7 +12954,7 @@
         <v>20375803</v>
       </c>
       <c r="F414" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="G414" t="str">
         <f t="shared" si="6"/>
@@ -12963,13 +12963,13 @@
     </row>
     <row r="415" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A415" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B415" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C415" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D415" s="3">
         <v>22876025</v>
@@ -12978,7 +12978,7 @@
         <v>22876275</v>
       </c>
       <c r="F415" s="1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="G415" t="str">
         <f t="shared" si="6"/>
@@ -12987,13 +12987,13 @@
     </row>
     <row r="416" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A416" s="1" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B416" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D416" s="3">
         <v>23563997</v>
@@ -13002,7 +13002,7 @@
         <v>23564326</v>
       </c>
       <c r="F416" s="1" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G416" t="str">
         <f t="shared" si="6"/>
@@ -13011,13 +13011,13 @@
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A417" s="1" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B417" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C417" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D417" s="3">
         <v>38757725</v>
@@ -13026,7 +13026,7 @@
         <v>38758112</v>
       </c>
       <c r="F417" s="1" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="G417" t="str">
         <f t="shared" si="6"/>
@@ -13035,13 +13035,13 @@
     </row>
     <row r="418" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A418" s="1" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B418" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C418" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D418" s="3">
         <v>55370708</v>
@@ -13050,7 +13050,7 @@
         <v>55370863</v>
       </c>
       <c r="F418" s="1" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G418" t="str">
         <f t="shared" si="6"/>
@@ -13059,13 +13059,13 @@
     </row>
     <row r="419" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A419" s="1" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B419" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C419" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D419" s="3">
         <v>55379519</v>
@@ -13074,7 +13074,7 @@
         <v>55379958</v>
       </c>
       <c r="F419" s="1" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="G419" t="str">
         <f t="shared" si="6"/>
@@ -13083,13 +13083,13 @@
     </row>
     <row r="420" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A420" s="1" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B420" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C420" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D420" s="3">
         <v>55382639</v>
@@ -13098,7 +13098,7 @@
         <v>55382877</v>
       </c>
       <c r="F420" s="1" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="G420" t="str">
         <f t="shared" si="6"/>
@@ -13107,13 +13107,13 @@
     </row>
     <row r="421" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A421" s="1" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B421" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C421" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D421" s="3">
         <v>56901630</v>
@@ -13122,7 +13122,7 @@
         <v>56901792</v>
       </c>
       <c r="F421" s="1" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="G421" t="str">
         <f t="shared" si="6"/>
@@ -13131,13 +13131,13 @@
     </row>
     <row r="422" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A422" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B422" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C422" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D422" s="3">
         <v>70946890</v>
@@ -13146,7 +13146,7 @@
         <v>70947123</v>
       </c>
       <c r="F422" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="G422" t="str">
         <f t="shared" si="6"/>
@@ -13155,13 +13155,13 @@
     </row>
     <row r="423" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A423" s="1" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B423" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C423" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D423" s="3">
         <v>70984269</v>
@@ -13170,7 +13170,7 @@
         <v>70984560</v>
       </c>
       <c r="F423" s="1" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="G423" t="str">
         <f t="shared" si="6"/>
@@ -13179,13 +13179,13 @@
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A424" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B424" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C424" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D424" s="3">
         <v>92607187</v>
@@ -13194,7 +13194,7 @@
         <v>92607387</v>
       </c>
       <c r="F424" s="1" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="G424" t="str">
         <f t="shared" si="6"/>
@@ -13203,13 +13203,13 @@
     </row>
     <row r="425" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A425" s="1" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B425" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C425" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D425" s="3">
         <v>97171939</v>
@@ -13218,7 +13218,7 @@
         <v>97172197</v>
       </c>
       <c r="F425" s="1" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="G425" t="str">
         <f t="shared" si="6"/>
@@ -13227,13 +13227,13 @@
     </row>
     <row r="426" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A426" s="1" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B426" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C426" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D426" s="3">
         <v>99986545</v>
@@ -13242,7 +13242,7 @@
         <v>99987001</v>
       </c>
       <c r="F426" s="1" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="G426" t="str">
         <f t="shared" si="6"/>
@@ -13251,13 +13251,13 @@
     </row>
     <row r="427" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A427" s="1" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B427" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C427" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D427" s="3">
         <v>116679722</v>
@@ -13266,7 +13266,7 @@
         <v>116679936</v>
       </c>
       <c r="F427" s="1" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="G427" t="str">
         <f t="shared" si="6"/>
@@ -13275,13 +13275,13 @@
     </row>
     <row r="428" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A428" s="1" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B428" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C428" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D428" s="3">
         <v>143667537</v>
@@ -13290,7 +13290,7 @@
         <v>143667764</v>
       </c>
       <c r="F428" s="1" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G428" t="str">
         <f t="shared" si="6"/>
@@ -13299,13 +13299,13 @@
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A429" s="1" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B429" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C429" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D429" s="3">
         <v>145105504</v>
@@ -13314,7 +13314,7 @@
         <v>145106417</v>
       </c>
       <c r="F429" s="1" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="G429" t="str">
         <f t="shared" si="6"/>
@@ -13323,13 +13323,13 @@
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A430" s="1" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B430" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C430" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D430" s="3">
         <v>97506250</v>
@@ -13338,7 +13338,7 @@
         <v>97506398</v>
       </c>
       <c r="F430" s="1" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="G430" t="str">
         <f t="shared" si="6"/>
@@ -13347,13 +13347,13 @@
     </row>
     <row r="431" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A431" s="1" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B431" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C431" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D431" s="3">
         <v>41166232</v>
@@ -13362,7 +13362,7 @@
         <v>41166296</v>
       </c>
       <c r="F431" s="1" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="G431" t="str">
         <f t="shared" si="6"/>
@@ -13371,13 +13371,13 @@
     </row>
     <row r="432" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A432" s="1" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D432" s="3">
         <v>55370371</v>
@@ -13386,7 +13386,7 @@
         <v>55370440</v>
       </c>
       <c r="F432" s="1" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G432" t="str">
         <f t="shared" si="6"/>
@@ -13395,13 +13395,13 @@
     </row>
     <row r="433" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A433" s="1" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D433" s="3">
         <v>124332801</v>
@@ -13410,7 +13410,7 @@
         <v>124332922</v>
       </c>
       <c r="F433" s="1" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="G433" t="str">
         <f t="shared" si="6"/>
@@ -13419,13 +13419,13 @@
     </row>
     <row r="434" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A434" s="1" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B434" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C434" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D434" s="3">
         <v>20375518</v>
@@ -13434,7 +13434,7 @@
         <v>20375639</v>
       </c>
       <c r="F434" s="1" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="G434" t="str">
         <f t="shared" si="6"/>
@@ -13443,13 +13443,13 @@
     </row>
     <row r="435" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A435" s="1" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B435" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C435" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D435" s="3">
         <v>1042341</v>
@@ -13458,7 +13458,7 @@
         <v>1042870</v>
       </c>
       <c r="F435" s="1" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="G435" t="str">
         <f t="shared" si="6"/>
@@ -13467,13 +13467,13 @@
     </row>
     <row r="436" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A436" s="1" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C436" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D436" s="3">
         <v>13323138</v>
@@ -13482,7 +13482,7 @@
         <v>13323350</v>
       </c>
       <c r="F436" s="1" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="G436" t="str">
         <f t="shared" si="6"/>
@@ -13491,13 +13491,13 @@
     </row>
     <row r="437" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A437" s="1" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C437" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D437" s="3">
         <v>14346833</v>
@@ -13506,7 +13506,7 @@
         <v>14347127</v>
       </c>
       <c r="F437" s="1" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G437" t="str">
         <f t="shared" si="6"/>
@@ -13515,13 +13515,13 @@
     </row>
     <row r="438" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A438" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B438" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C438" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D438" s="3">
         <v>19788614</v>
@@ -13530,7 +13530,7 @@
         <v>19788770</v>
       </c>
       <c r="F438" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G438" t="str">
         <f t="shared" si="6"/>
@@ -13539,13 +13539,13 @@
     </row>
     <row r="439" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A439" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B439" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C439" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D439" s="3">
         <v>19789005</v>
@@ -13554,7 +13554,7 @@
         <v>19789196</v>
       </c>
       <c r="F439" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G439" t="str">
         <f t="shared" si="6"/>
@@ -13563,13 +13563,13 @@
     </row>
     <row r="440" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A440" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B440" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C440" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D440" s="3">
         <v>27690516</v>
@@ -13578,7 +13578,7 @@
         <v>27690698</v>
       </c>
       <c r="F440" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="G440" t="str">
         <f t="shared" si="6"/>
@@ -13587,13 +13587,13 @@
     </row>
     <row r="441" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A441" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B441" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C441" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D441" s="3">
         <v>36986083</v>
@@ -13602,7 +13602,7 @@
         <v>36986751</v>
       </c>
       <c r="F441" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="G441" t="str">
         <f t="shared" si="6"/>
@@ -13611,13 +13611,13 @@
     </row>
     <row r="442" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A442" s="1" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B442" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C442" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D442" s="3">
         <v>36986898</v>
@@ -13626,7 +13626,7 @@
         <v>36987141</v>
       </c>
       <c r="F442" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="G442" t="str">
         <f t="shared" si="6"/>
@@ -13635,13 +13635,13 @@
     </row>
     <row r="443" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A443" s="1" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B443" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C443" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D443" s="3">
         <v>100616259</v>
@@ -13650,7 +13650,7 @@
         <v>100616670</v>
       </c>
       <c r="F443" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="G443" t="str">
         <f t="shared" si="6"/>
@@ -13659,13 +13659,13 @@
     </row>
     <row r="444" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A444" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B444" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C444" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D444" s="3">
         <v>120507170</v>
@@ -13674,7 +13674,7 @@
         <v>120507467</v>
       </c>
       <c r="F444" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G444" t="str">
         <f t="shared" si="6"/>
@@ -13683,13 +13683,13 @@
     </row>
     <row r="445" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A445" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B445" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C445" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D445" s="3">
         <v>126778344</v>
@@ -13698,7 +13698,7 @@
         <v>126778602</v>
       </c>
       <c r="F445" s="1" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G445" t="str">
         <f t="shared" si="6"/>
@@ -13707,13 +13707,13 @@
     </row>
     <row r="446" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A446" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B446" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C446" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D446" s="3">
         <v>127265692</v>
@@ -13722,7 +13722,7 @@
         <v>127265900</v>
       </c>
       <c r="F446" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G446" t="str">
         <f t="shared" si="6"/>
@@ -13731,13 +13731,13 @@
     </row>
     <row r="447" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A447" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B447" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C447" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D447" s="3">
         <v>132650647</v>
@@ -13746,7 +13746,7 @@
         <v>132650877</v>
       </c>
       <c r="F447" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="G447" t="str">
         <f t="shared" si="6"/>
@@ -13755,13 +13755,13 @@
     </row>
     <row r="448" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A448" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B448" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C448" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D448" s="3">
         <v>132651024</v>
@@ -13770,7 +13770,7 @@
         <v>132651124</v>
       </c>
       <c r="F448" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="G448" t="str">
         <f t="shared" si="6"/>
@@ -13779,13 +13779,13 @@
     </row>
     <row r="449" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A449" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B449" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C449" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D449" s="3">
         <v>133771498</v>
@@ -13794,7 +13794,7 @@
         <v>133771758</v>
       </c>
       <c r="F449" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G449" t="str">
         <f t="shared" si="6"/>
@@ -13803,13 +13803,13 @@
     </row>
     <row r="450" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A450" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B450" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C450" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D450" s="3">
         <v>135462414</v>
@@ -13818,7 +13818,7 @@
         <v>135462593</v>
       </c>
       <c r="F450" s="1" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="G450" t="str">
         <f t="shared" si="6"/>
@@ -13827,13 +13827,13 @@
     </row>
     <row r="451" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A451" s="1" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C451" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D451" s="3">
         <v>139428562</v>
@@ -13842,7 +13842,7 @@
         <v>139428679</v>
       </c>
       <c r="F451" s="1" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="G451" t="str">
         <f t="shared" ref="G451:G452" si="7">C451&amp;":"&amp;D451&amp;"-"&amp;E451</f>
@@ -13851,13 +13851,13 @@
     </row>
     <row r="452" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A452" s="1" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C452" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D452" s="3">
         <v>21974677</v>
@@ -13866,7 +13866,7 @@
         <v>21974779</v>
       </c>
       <c r="F452" s="1" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="G452" t="str">
         <f t="shared" si="7"/>

</xml_diff>